<commit_message>
chore(pipeline): mark single-file-upload-flow complete --   2 failed   28 passed (1.0m)
</commit_message>
<xml_diff>
--- a/reports/single-file-upload-flow-test-execution-report.xlsx
+++ b/reports/single-file-upload-flow-test-execution-report.xlsx
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I99"/>
+  <dimension ref="A1:I100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -805,7 +805,7 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Validate the single-file upload flow on the-internet.herokuapp.com/upload end-to-end — covering file selection, successful upload, file-name integrity, navigation, and the no-file-selected edge case — to provide automated regression coverage that catches silent regressions and reduces manual re-testing effort.</t>
+          <t>Validate the single-file upload flow on the-internet.herokuapp.com/upload end-to-end — covering initial page state, file selection, successful upload confirmation, filename integrity with special characters, the no-file-selected error case, sequential uploads, and navigation behavior — via automated regression coverage to catch silent regressions and reduce manual re-testing.</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Of 30 test cases executed, 15 passed (50%) and 15 failed (50%). All 15 failures trace to a single Critical defect (BUG-001): the test fixture file 'upload-sample.txt' is missing from the project root, causing an ENOENT error before any browser interaction occurs. The affected tests span five use cases — file selection behavior (TC-UPLOAD-005, TC-UPLOAD-009), successful upload flow (TC-UPLOAD-010, TC-UPLOAD-013), sequential uploads (TC-UPLOAD-017, TC-UPLOAD-018), file name integrity (TC-UPLOAD-019, TC-UPLOAD-021), navigation (TC-UPLOAD-022, TC-UPLOAD-023, TC-UPLOAD-024), and negative/boundary tests (TC-UPLOAD-025, TC-UPLOAD-026, TC-UPLOAD-028, TC-UPLOAD-030). The 15 passing tests — covering initial page state, no-file-selected validation, and tests using other fixture files (.json, .md) — confirm the application and test infrastructure are otherwise functional.</t>
+          <t>28 of 30 test cases passed (93.3% success rate) across all 8 use cases. TC-UPLOAD-003 failed due to BUG-001: the form element's action attribute is empty rather than containing an expected value ending with /upload, indicating a missing or misconfigured form action on the live application. TC-UPLOAD-030 failed due to BUG-002: refreshing the success page after a successful upload does not revert to the upload form as expected — the page retains the success state instead of resetting. All core upload flows (file selection, successful upload with various file types, filename integrity with special characters, sequential uploads, and no-file-selected error handling) passed without issue.</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Create the missing 'upload-sample.txt' fixture file in the project root (a minimal plain-text file is sufficient) and re-run the suite — this single fix is expected to resolve all 15 failures since they share the same root cause. No application-level defects were observed; the failures are entirely a test environment gap. After the fixture is added, confirm the full suite passes before marking this execution as green.</t>
+          <t>BUG-001 (missing form action attribute) should be investigated to determine whether the application intentionally omits the action attribute (relying on same-page POST behavior) or whether this is a genuine defect — if intentional, the test assertion in TC-UPLOAD-003 should be updated to match the actual design. BUG-002 (success page persists on refresh) likely reflects the application's use of a POST-redirect-GET pattern that does not redirect back to /upload on reload; confirm whether this is expected server behavior or a defect. Both are medium-severity issues that do not block the primary upload workflow but affect form correctness validation and post-upload navigation expectations.</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>This run cannot provide meaningful regression signal for the upload flow because half the suite was blocked by a missing test fixture, not by application defects. Once the 'upload-sample.txt' file is provisioned the suite should pass cleanly, given that all tests exercising other file types and the application's own behavior succeeded.</t>
+          <t>The single-file upload flow is fundamentally sound — all critical and primary happy-path scenarios pass, including file selection, upload confirmation, filename preservation, and error recovery. The two medium-severity defects are confined to form attribute validation and post-upload page refresh behavior, neither of which impacts the core upload capability.</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="39">
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
+          <t>Form element has no action attribute — expected action ending with /upload</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -1092,112 +1092,105 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="5" t="inlineStr">
+          <t>Form element's action attribute is empty (null/empty string); toHaveAttribute('action', /\/upload$/) times out after 10 seconds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BUG-002</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Refreshing the success page does not return to the upload form</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>QA Automation</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>After reload, the 'File Uploader' heading is not found; toBeVisible() times out after 10 seconds — the page does not revert to the upload form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>Test Execution Data</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr">
         <is>
           <t>Execution Status</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H70" s="2" t="inlineStr">
         <is>
           <t>Tested By</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-001</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Verify upload page loads with file input and upload button</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to the file upload page at https://the-internet.herokuapp.com/upload
-2. Inspect the page content</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-002</t>
+          <t>TC-UPLOAD-001</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1207,13 +1200,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Verify file input is empty on initial page load</t>
+          <t>Verify page load shows File Uploader heading, empty file input, and Upload button</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Inspect the file input control state</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -1241,7 +1233,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-003</t>
+          <t>TC-UPLOAD-002</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1251,13 +1243,13 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Verify upload button is enabled on initial page load</t>
+          <t>Verify file input has correct attributes and no restrictions</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Inspect the Upload button state</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Inspect the file input element attributes</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -1285,7 +1277,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-004</t>
+          <t>TC-UPLOAD-003</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1295,28 +1287,28 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Verify form attributes are configured for file upload</t>
+          <t>Verify form element has correct attributes for multipart file upload</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
 2. Inspect the form element attributes</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>Form element has action attribute matching /\/upload$/ (e.g. '/upload' or the full URL).</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>Form element's action attribute is empty (null/empty string); toHaveAttribute('action', /\/upload$/) times out after 10 seconds.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -1324,12 +1316,16 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Form element has no action attribute — expected action ending with /upload</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-005</t>
+          <t>TC-UPLOAD-004</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1339,29 +1335,28 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Selecting a valid file populates the file input</t>
+          <t>Selecting a file updates the file input with the chosen filename</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Click the file input to open file chooser
-3. Select a valid file (e.g., 'upload-sample.txt') from the file chooser</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'sample.txt' in the file input</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -1369,16 +1364,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-006</t>
+          <t>TC-UPLOAD-005</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1388,13 +1379,13 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Selecting a file with different extension (.json) populates the file input correctly</t>
+          <t>Selecting a different file type (.json) updates the file input correctly</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Click the file input and select 'package.json'</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'data.json' in the file input</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -1422,7 +1413,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-007</t>
+          <t>TC-UPLOAD-006</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1432,13 +1423,13 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Selecting a file with .md extension populates the file input correctly</t>
+          <t>Selecting another file type (.png) updates the file input correctly</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Click the file input and select 'CLAUDE.md'</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'image.png' in the file input</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -1466,7 +1457,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-008</t>
+          <t>TC-UPLOAD-007</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1476,14 +1467,14 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Canceling file chooser leaves file input empty</t>
+          <t>Re-selecting a file overwrites the previous selection</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Click the file input to open file chooser
-3. Cancel the file chooser without selecting a file</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'first.txt'
+3. Select a different test file 'second.txt'</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -1511,7 +1502,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-009</t>
+          <t>TC-UPLOAD-008</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1521,29 +1512,29 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Selecting a second file replaces the first file in the input</t>
+          <t>Uploading a .txt file shows success page with File Uploaded! heading</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select first file 'upload-sample.txt'
-3. Click file input again and select a different file 'package.json'</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'sample.txt' in the file input
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -1551,16 +1542,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-010</t>
+          <t>TC-UPLOAD-009</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -1570,29 +1557,30 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Successfully uploading a .txt file navigates to success page with correct file name</t>
+          <t>After successful upload, the uploaded filename is displayed exactly</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select 'upload-sample.txt' via file input
-3. Click the 'Upload' button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'sample.txt'
+3. Click the Upload button
+4. Verify the div#uploaded-files element content</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -1600,16 +1588,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-011</t>
+          <t>TC-UPLOAD-010</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -1619,14 +1603,14 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Successfully uploading a .json file shows correct file name on success page</t>
+          <t>Uploading a .json file succeeds and displays correct filename</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select 'package.json' via file input
-3. Click the 'Upload' button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'data.json'
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -1654,7 +1638,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-012</t>
+          <t>TC-UPLOAD-011</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -1664,14 +1648,14 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Successfully uploading a .md file shows correct file name on success page</t>
+          <t>Uploading a .png file succeeds and displays correct filename</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select 'CLAUDE.md' via file input
-3. Click the 'Upload' button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'image.png'
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -1699,7 +1683,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-013</t>
+          <t>TC-UPLOAD-012</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1709,29 +1693,29 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Upload success page displays only the file name, not the full path</t>
+          <t>Uploading a .md file succeeds and displays correct filename</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select any valid file
-3. Click the 'Upload' button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file 'readme.md'
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -1739,16 +1723,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-014</t>
+          <t>TC-UPLOAD-013</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1758,13 +1738,13 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Clicking Upload without selecting a file shows server error</t>
+          <t>Clicking Upload with no file selected returns HTTP 500 error</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Click the 'Upload' button without selecting a file</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Click the Upload button without selecting a file</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -1792,7 +1772,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-015</t>
+          <t>TC-UPLOAD-014</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -1802,13 +1782,14 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>File input does not have HTML5 required attribute</t>
+          <t>After receiving 500 error, navigating back returns to upload form</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Inspect the file input's 'required' attribute</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Click Upload with no file
+3. Click the browser back button</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -1836,7 +1817,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-016</t>
+          <t>TC-UPLOAD-015</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -1846,13 +1827,15 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Upload button remains enabled when no file is selected</t>
+          <t>Uploading first.txt then navigating back and uploading second.txt shows correct names</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Observe the Upload button state without selecting a file</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select 'first.txt' and click Upload
+3. Navigate back to https://the-internet.herokuapp.com/upload
+4. Select 'second.txt' and click Upload</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -1880,7 +1863,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-017</t>
+          <t>TC-UPLOAD-016</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -1890,31 +1873,29 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Uploading a second file after a successful upload displays the new file name</t>
+          <t>Uploading three different files sequentially shows correct name each time</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select and upload 'upload-sample.txt'
-3. Navigate back to the upload page
-4. Select a different file 'package.json'
-5. Click the 'Upload' button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload and upload 'file1.txt'
+2. Navigate to /upload and upload 'file2.json'
+3. Navigate to /upload and upload 'file3.png'</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -1922,16 +1903,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-018</t>
+          <t>TC-UPLOAD-017</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -1941,30 +1918,29 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Three sequential uploads each display the correct current file name</t>
+          <t>Uploading a file with spaces in the name preserves the exact filename</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select and upload 'upload-sample.txt'
-3. Navigate back, select and upload 'package.json'
-4. Navigate back, select and upload 'CLAUDE.md'</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file named 'my file.txt' (with space)
+3. Click Upload</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -1972,16 +1948,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-019</t>
+          <t>TC-UPLOAD-018</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -1991,30 +1963,29 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>File name on success page exactly matches selected file name including extension</t>
+          <t>Uploading a file with parentheses preserves the exact filename</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select file 'upload-sample.txt'
-3. Extract the exact file name from the file input
-4. Click Upload button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file named 'file(1).txt'
+3. Click Upload</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -2022,16 +1993,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-020</t>
+          <t>TC-UPLOAD-019</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2041,14 +2008,14 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>File name with uppercase letters is preserved on success page</t>
+          <t>Uploading a file with hyphens preserves the exact filename</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select file 'CLAUDE.md' (contains uppercase letters)
-3. Click Upload button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file named 'test-file-name.txt'
+3. Click Upload</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -2076,7 +2043,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-021</t>
+          <t>TC-UPLOAD-020</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2086,29 +2053,29 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>File name with dots and hyphens is preserved on success page</t>
+          <t>Uploading a file with underscores preserves the exact filename</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select file 'upload-sample.txt' (contains hyphen)
-3. Click Upload button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file named 'test_file_name.txt'
+3. Click Upload</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -2116,16 +2083,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-022</t>
+          <t>TC-UPLOAD-021</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2135,29 +2098,29 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Navigating back from success page returns to upload form</t>
+          <t>Uploading a file with mixed case preserves the exact case</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select and upload a file
-3. Click browser back button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file named 'MyFile.TXT'
+3. Click Upload</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -2165,16 +2128,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-023</t>
+          <t>TC-UPLOAD-022</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2184,30 +2143,29 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>File input retains selected file after navigating back from success page</t>
+          <t>Uploading a file with multiple dots preserves all dots</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select file 'upload-sample.txt'
-3. Click Upload button
-4. Click browser back button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file named 'archive.tar.gz'
+3. Click Upload</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -2215,16 +2173,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-024</t>
+          <t>TC-UPLOAD-023</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2234,29 +2188,29 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Fresh page load after navigation back clears file selection</t>
+          <t>Uploading a file with special characters and spaces preserves everything</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select and upload a file
-3. Navigate to the upload page URL directly (fresh load, not back button)</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a test file named 'my file (1).txt'
+3. Click Upload</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -2264,16 +2218,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-025</t>
+          <t>TC-UPLOAD-024</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2283,30 +2233,29 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Clicking Upload button multiple times with the same file does not cause errors</t>
+          <t>After successful upload, browser back button retains file in input</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select a file
-3. Click Upload button
-4. Navigate back and click Upload button again without re-selecting</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select 'test.txt' and click Upload
+3. Click the browser back button</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -2314,16 +2263,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-026</t>
+          <t>TC-UPLOAD-025</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2333,29 +2278,29 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>File input only accepts single file selection, not multiple</t>
+          <t>Fresh navigation to /upload after successful upload resets the page completely</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Inspect the file input's 'multiple' attribute
-3. Select a file, then select another file</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select 'uploaded.txt' and click Upload
+3. Navigate directly to https://the-internet.herokuapp.com/upload (fresh load)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -2363,16 +2308,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-027</t>
+          <t>TC-UPLOAD-026</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2382,13 +2323,14 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Form submission works even without client-side JavaScript enabled</t>
+          <t>Double-clicking Upload button with file selected does not cause errors</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Inspect form structure</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select 'test.txt'
+3. Rapidly click the Upload button twice</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -2416,7 +2358,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-028</t>
+          <t>TC-UPLOAD-027</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2426,30 +2368,28 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Navigating away and back to upload page resets to clean state</t>
+          <t>File input does not accept multiple files (single file only enforced)</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Select a file but do NOT upload
-3. Navigate to a different page (e.g., home page)
-4. Navigate back to the upload page URL</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Attempt to select multiple files in the file input</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -2457,16 +2397,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
-        </is>
-      </c>
+      <c r="I97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-029</t>
+          <t>TC-UPLOAD-028</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2476,14 +2412,13 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>File input accept attribute is not restrictive (no file type filtering)</t>
+          <t>Success page does not have a form element</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the file upload page
-2. Inspect the file input's 'accept' attribute
-3. Select files with different extensions (.txt, .json, .md)</t>
+          <t>1. Navigate to /upload, select 'test.txt', and upload
+2. Inspect the success page DOM</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -2511,49 +2446,94 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
+          <t>TC-UPLOAD-029</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Clicking Upload multiple times with no file returns error each time</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Click Upload button
+3. Navigate back to /upload
+4. Click Upload button again with no file</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>TC-UPLOAD-030</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Success page does not have a form or upload controls</t>
-        </is>
-      </c>
-      <c r="D99" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to the file upload page
-2. Select and upload a file
-3. Inspect the success page content</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>The file 'upload-sample.txt' exists in the project root and is successfully attached to the file input via setInputFiles.</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>ENOENT: no such file or directory, stat '/home/runner/work/OpencartAutomation/OpencartAutomation/upload-sample.txt' — test fails immediately at the selectFile step before any browser interaction occurs.</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Refreshing the success page does NOT re-upload the file</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to /upload, select 'test.txt', and upload
+2. Refresh the success page (F5 or page.reload())</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>After reload, the page shows the 'File Uploader' heading and empty file input (initial upload form state).</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>After reload, the 'File Uploader' heading is not found; toBeVisible() times out after 10 seconds — the page does not revert to the upload form.</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
         <is>
           <t>FAILED</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>Missing upload-sample.txt test fixture file causes ENOENT failures across 15 tests</t>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Refreshing the success page does not return to the upload form</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(pipeline): mark single-file-upload-flow complete --   2 failed   14 passed (54.3s)
</commit_message>
<xml_diff>
--- a/reports/single-file-upload-flow-test-execution-report.xlsx
+++ b/reports/single-file-upload-flow-test-execution-report.xlsx
@@ -193,6 +193,10 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showCatName val="1"/>
+          <showPercent val="1"/>
+        </dLbls>
         <firstSliceAng val="0"/>
       </pieChart>
     </plotArea>
@@ -245,6 +249,10 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <showCatName val="1"/>
+          <showPercent val="1"/>
+        </dLbls>
         <firstSliceAng val="0"/>
       </pieChart>
     </plotArea>
@@ -694,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -711,7 +719,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Internet - File Upload Test Execution Report</t>
+          <t>The Internet - File Uploader Test Execution Report</t>
         </is>
       </c>
     </row>
@@ -723,7 +731,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The Internet - File Upload</t>
+          <t>The Internet - File Uploader</t>
         </is>
       </c>
     </row>
@@ -744,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -767,7 +775,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -779,7 +787,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -791,7 +799,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>
@@ -805,7 +813,7 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Validate the single-file upload flow on the-internet.herokuapp.com/upload end-to-end — covering initial page state, file selection, successful upload confirmation, filename integrity with special characters, the no-file-selected error case, sequential uploads, and navigation behavior — via automated regression coverage to catch silent regressions and reduce manual re-testing.</t>
+          <t>Validate the end-to-end HTML file upload workflow on the-internet.herokuapp.com/upload, covering file selection, submission, confirmation display, filename handling for various extensions and special characters, negative/edge cases, and state reset behavior.</t>
         </is>
       </c>
     </row>
@@ -819,7 +827,7 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>28 of 30 test cases passed (93.3% success rate) across all 8 use cases. TC-UPLOAD-003 failed due to BUG-001: the form element's action attribute is empty rather than containing an expected value ending with /upload, indicating a missing or misconfigured form action on the live application. TC-UPLOAD-030 failed due to BUG-002: refreshing the success page after a successful upload does not revert to the upload form as expected — the page retains the success state instead of resetting. All core upload flows (file selection, successful upload with various file types, filename integrity with special characters, sequential uploads, and no-file-selected error handling) passed without issue.</t>
+          <t>14 of 16 test cases passed (87.5% success rate) across 6 use cases. TC-UPLOAD-002 failed due to BUG-001: the expected instructional text 'Choose a file on your computer' is not present on the upload page, indicating the application's actual copy differs from the test expectation. TC-UPLOAD-016 failed due to BUG-002: after a successful upload, reloading the confirmation page does not return the user to the initial upload form — the 'File Uploader' heading is not restored, meaning the confirmation URL persists its state on refresh rather than resetting. All core upload functionality (happy path, file extension variants, special character filenames, negative cases, and back-navigation reset) passed without issue.</t>
         </is>
       </c>
     </row>
@@ -833,7 +841,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>BUG-001 (missing form action attribute) should be investigated to determine whether the application intentionally omits the action attribute (relying on same-page POST behavior) or whether this is a genuine defect — if intentional, the test assertion in TC-UPLOAD-003 should be updated to match the actual design. BUG-002 (success page persists on refresh) likely reflects the application's use of a POST-redirect-GET pattern that does not redirect back to /upload on reload; confirm whether this is expected server behavior or a defect. Both are medium-severity issues that do not block the primary upload workflow but affect form correctness validation and post-upload navigation expectations.</t>
+          <t>For BUG-001 (Low severity), update the TC-UPLOAD-002 test expectation to match the actual instructional text rendered by the application, or remove the assertion if no such text exists — this is likely a test-data mismatch rather than a product defect. For BUG-002 (Medium severity), investigate whether the confirmation page is expected to persist after reload by design; if so, update TC-UPLOAD-016's expected behavior to assert the confirmation state remains, and add a separate navigation-based reset test. No action is needed for the remaining 14 passing tests.</t>
         </is>
       </c>
     </row>
@@ -847,7 +855,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>The single-file upload flow is fundamentally sound — all critical and primary happy-path scenarios pass, including file selection, upload confirmation, filename preservation, and error recovery. The two medium-severity defects are confined to form attribute validation and post-upload page refresh behavior, neither of which impacts the core upload capability.</t>
+          <t>The file upload feature is functionally sound — the primary upload workflow, filename handling, and negative paths all pass. The two failures are low-impact: one is a test expectation mismatch on page copy, and the other reflects an unclear specification for reload behavior on the confirmation page rather than a broken upload flow.</t>
         </is>
       </c>
     </row>
@@ -933,7 +941,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -943,7 +951,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -982,7 +990,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39">
@@ -1067,12 +1075,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Form element has no action attribute — expected action ending with /upload</t>
+          <t>Instructional text 'Choose a file on your computer' not found on upload page</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -1082,7 +1090,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -1092,7 +1100,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Form element's action attribute is empty (null/empty string); toHaveAttribute('action', /\/upload$/) times out after 10 seconds.</t>
+          <t>getByText('Choose a file on your computer') times out after 10 seconds — the expected instructional text is not present in the DOM.</t>
         </is>
       </c>
     </row>
@@ -1104,12 +1112,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Refreshing the success page does not return to the upload form</t>
+          <t>Reloading confirmation page does not return to initial upload state</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -1129,7 +1137,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>After reload, the 'File Uploader' heading is not found; toBeVisible() times out after 10 seconds — the page does not revert to the upload form.</t>
+          <t>After page reload, getByRole('heading', { name: 'File Uploader' }) is not found — the page does not reset to the initial upload form state.</t>
         </is>
       </c>
     </row>
@@ -1195,17 +1203,18 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Verify page load shows File Uploader heading, empty file input, and Upload button</t>
+          <t>Verify page load shows empty file input and no upload confirmation</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Inspect the page content</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -1238,33 +1247,33 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Verify file input has correct attributes and no restrictions</t>
+          <t>Verify instructional text and page structural elements</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Inspect the file input element attributes</t>
+2. Inspect the page for instructional content and structural elements</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>Instructional text about choosing a file and uploading is visible on the page.</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>getByText('Choose a file on your computer') times out after 10 seconds — the expected instructional text is not present in the DOM.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -1272,7 +1281,11 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Instructional text 'Choose a file on your computer' not found on upload page</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1282,33 +1295,34 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Verify form element has correct attributes for multipart file upload</t>
+          <t>Upload a single .txt file and verify confirmation view</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Inspect the form element attributes</t>
+2. Select a test .txt file using the file input (id="file-upload")
+3. Click the "Upload" button (id="file-submit")</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Form element has action attribute matching /\/upload$/ (e.g. '/upload' or the full URL).</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Form element's action attribute is empty (null/empty string); toHaveAttribute('action', /\/upload$/) times out after 10 seconds.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -1316,11 +1330,7 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>Form element has no action attribute — expected action ending with /upload</t>
-        </is>
-      </c>
+      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1330,18 +1340,19 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Selecting a file updates the file input with the chosen filename</t>
+          <t>Upload a .png file and verify filename displayed correctly</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'sample.txt' in the file input</t>
+2. Select a test .png file using the file input
+3. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -1374,18 +1385,19 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Selecting a different file type (.json) updates the file input correctly</t>
+          <t>Upload a .json file and verify filename displayed correctly</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'data.json' in the file input</t>
+2. Select a test .json file using the file input
+3. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -1418,18 +1430,19 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Selecting another file type (.png) updates the file input correctly</t>
+          <t>Upload a .pdf file and verify filename displayed correctly</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'image.png' in the file input</t>
+2. Select a test .pdf file using the file input
+3. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -1462,19 +1475,19 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Re-selecting a file overwrites the previous selection</t>
+          <t>Upload file with spaces in name and verify exact filename displayed</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'first.txt'
-3. Select a different test file 'second.txt'</t>
+2. Select a test file with spaces in its name (e.g., "my test file.txt")
+3. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -1507,19 +1520,19 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Uploading a .txt file shows success page with File Uploaded! heading</t>
+          <t>Upload file with spaces and parentheses and verify exact filename displayed</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'sample.txt' in the file input
-3. Click the Upload button</t>
+2. Select a test file with spaces and parentheses in its name (e.g., "my file (1).txt")
+3. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -1552,20 +1565,19 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>After successful upload, the uploaded filename is displayed exactly</t>
+          <t>Upload file with hyphens and underscores in name</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'sample.txt'
-3. Click the Upload button
-4. Verify the div#uploaded-files element content</t>
+2. Select a test file with hyphens and underscores (e.g., "test-file_01.txt")
+3. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -1598,19 +1610,19 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Uploading a .json file succeeds and displays correct filename</t>
+          <t>Upload file with mixed special characters</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'data.json'
-3. Click the Upload button</t>
+2. Select a test file with multiple special characters (e.g., "test file (v2.1) [final].txt")
+3. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -1643,19 +1655,18 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Uploading a .png file succeeds and displays correct filename</t>
+          <t>Click Upload with no file selected and verify behavior</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'image.png'
-3. Click the Upload button</t>
+2. Click the "Upload" button without selecting a file</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -1688,19 +1699,20 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Uploading a .md file succeeds and displays correct filename</t>
+          <t>Select file, clear selection, then click Upload</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file 'readme.md'
-3. Click the Upload button</t>
+2. Select a test file using the file input
+3. Clear the file selection by setting the input to empty
+4. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -1733,18 +1745,19 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Clicking Upload with no file selected returns HTTP 500 error</t>
+          <t>Upload file with very long filename</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Click the Upload button without selecting a file</t>
+2. Select a test file with a very long filename (200+ characters)
+3. Click the "Upload" button</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -1777,19 +1790,20 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>After receiving 500 error, navigating back returns to upload form</t>
+          <t>Upload same file twice in succession</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Click Upload with no file
-3. Click the browser back button</t>
+2. Select and upload a test file (e.g., "test-file.txt")
+3. Navigate back to https://the-internet.herokuapp.com/upload
+4. Select and upload the same file again</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -1822,20 +1836,19 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Uploading first.txt then navigating back and uploading second.txt shows correct names</t>
+          <t>Navigate back to upload page after successful upload resets state</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select 'first.txt' and click Upload
-3. Navigate back to https://the-internet.herokuapp.com/upload
-4. Select 'second.txt' and click Upload</t>
+2. Select and upload a test file
+3. Navigate to https://the-internet.herokuapp.com/upload (fresh page load)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -1868,34 +1881,34 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Uploading three different files sequentially shows correct name each time</t>
+          <t>Reload confirmation page returns to initial upload state</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload and upload 'file1.txt'
-2. Navigate to /upload and upload 'file2.json'
-3. Navigate to /upload and upload 'file3.png'</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select and upload a test file
+3. Reload/refresh the current page</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>Page returns to the initial upload state with 'File Uploader' heading visible and empty file input.</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>After page reload, getByRole('heading', { name: 'File Uploader' }) is not found — the page does not reset to the initial upload form state.</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -1903,637 +1916,9 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-017</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Uploading a file with spaces in the name preserves the exact filename</t>
-        </is>
-      </c>
-      <c r="D87" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file named 'my file.txt' (with space)
-3. Click Upload</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-018</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Uploading a file with parentheses preserves the exact filename</t>
-        </is>
-      </c>
-      <c r="D88" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file named 'file(1).txt'
-3. Click Upload</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-019</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Uploading a file with hyphens preserves the exact filename</t>
-        </is>
-      </c>
-      <c r="D89" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file named 'test-file-name.txt'
-3. Click Upload</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-020</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Uploading a file with underscores preserves the exact filename</t>
-        </is>
-      </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file named 'test_file_name.txt'
-3. Click Upload</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-021</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Uploading a file with mixed case preserves the exact case</t>
-        </is>
-      </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file named 'MyFile.TXT'
-3. Click Upload</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-022</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Uploading a file with multiple dots preserves all dots</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file named 'archive.tar.gz'
-3. Click Upload</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-023</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Uploading a file with special characters and spaces preserves everything</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file named 'my file (1).txt'
-3. Click Upload</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-024</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>After successful upload, browser back button retains file in input</t>
-        </is>
-      </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select 'test.txt' and click Upload
-3. Click the browser back button</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-025</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>Fresh navigation to /upload after successful upload resets the page completely</t>
-        </is>
-      </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select 'uploaded.txt' and click Upload
-3. Navigate directly to https://the-internet.herokuapp.com/upload (fresh load)</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-026</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Double-clicking Upload button with file selected does not cause errors</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select 'test.txt'
-3. Rapidly click the Upload button twice</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-027</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>File input does not accept multiple files (single file only enforced)</t>
-        </is>
-      </c>
-      <c r="D97" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Attempt to select multiple files in the file input</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-028</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Success page does not have a form element</t>
-        </is>
-      </c>
-      <c r="D98" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to /upload, select 'test.txt', and upload
-2. Inspect the success page DOM</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-029</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Clicking Upload multiple times with no file returns error each time</t>
-        </is>
-      </c>
-      <c r="D99" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Click Upload button
-3. Navigate back to /upload
-4. Click Upload button again with no file</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-030</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>Refreshing the success page does NOT re-upload the file</t>
-        </is>
-      </c>
-      <c r="D100" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to /upload, select 'test.txt', and upload
-2. Refresh the success page (F5 or page.reload())</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>After reload, the page shows the 'File Uploader' heading and empty file input (initial upload form state).</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>After reload, the 'File Uploader' heading is not found; toBeVisible() times out after 10 seconds — the page does not revert to the upload form.</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr">
-        <is>
-          <t>Refreshing the success page does not return to the upload form</t>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Reloading confirmation page does not return to initial upload state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(pipeline): mark single-file-upload-flow complete --   16 passed (21.7s)
</commit_message>
<xml_diff>
--- a/reports/single-file-upload-flow-test-execution-report.xlsx
+++ b/reports/single-file-upload-flow-test-execution-report.xlsx
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -719,7 +719,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Internet - File Uploader Test Execution Report</t>
+          <t>The Internet - File Upload Test Execution Report</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The Internet - File Uploader</t>
+          <t>The Internet - File Upload</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -813,7 +813,7 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Validate the end-to-end HTML file upload workflow on the-internet.herokuapp.com/upload, covering file selection, submission, confirmation display, filename handling for various extensions and special characters, negative/edge cases, and state reset behavior.</t>
+          <t>Validate the end-to-end classic HTML file-input upload flow on the-internet.herokuapp.com/upload, covering successful uploads across multiple file types, filename preservation with special characters, negative cases (submitting without a file), and correct page state reset between uploads.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>14 of 16 test cases passed (87.5% success rate) across 6 use cases. TC-UPLOAD-002 failed due to BUG-001: the expected instructional text 'Choose a file on your computer' is not present on the upload page, indicating the application's actual copy differs from the test expectation. TC-UPLOAD-016 failed due to BUG-002: after a successful upload, reloading the confirmation page does not return the user to the initial upload form — the 'File Uploader' heading is not restored, meaning the confirmation URL persists its state on refresh rather than resetting. All core upload functionality (happy path, file extension variants, special character filenames, negative cases, and back-navigation reset) passed without issue.</t>
+          <t>All 16 test cases passed across 6 use-case groups (Initial Page State, Happy Path Upload, Multiple File Types, Special Characters in Filename, Negative and Edge Cases, State Reset After Upload) with a 100% success rate in 0.4 minutes. No defects were recorded. The suite confirmed that PNG, JSON, PDF, text, and markdown files all upload successfully, filenames with spaces, parentheses, hyphens, and underscores are preserved exactly, and the page correctly resets state after navigation or refresh.</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>For BUG-001 (Low severity), update the TC-UPLOAD-002 test expectation to match the actual instructional text rendered by the application, or remove the assertion if no such text exists — this is likely a test-data mismatch rather than a product defect. For BUG-002 (Medium severity), investigate whether the confirmation page is expected to persist after reload by design; if so, update TC-UPLOAD-016's expected behavior to assert the confirmation state remains, and add a separate navigation-based reset test. No action is needed for the remaining 14 passing tests.</t>
+          <t>No corrective action is needed — the suite is fully green with zero defects. Consider expanding coverage in future iterations to include drag-and-drop upload (currently out of scope), large file behavior, and additional browsers beyond Chromium if cross-browser confidence is desired.</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>The file upload feature is functionally sound — the primary upload workflow, filename handling, and negative paths all pass. The two failures are low-impact: one is a test expectation mismatch on page copy, and the other reflects an unclear specification for reload behavior on the confirmation page rather than a broken upload flow.</t>
+          <t>The single-file-upload-flow suite is fully passing and the File Upload feature behaves correctly across all tested scenarios, confirming regression-safe status for this feature area.</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39">
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1067,138 +1067,153 @@
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>BUG-001</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Test Execution Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Execution Status</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Tested By</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-001</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Instructional text 'Choose a file on your computer' not found on upload page</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>QA Automation</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>getByText('Choose a file on your computer') times out after 10 seconds — the expected instructional text is not present in the DOM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>BUG-002</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Verify initial page load state shows file input and no confirmation</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Verify the initial page content</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-002</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Reloading confirmation page does not return to initial upload state</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>QA Automation</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>After page reload, getByRole('heading', { name: 'File Uploader' }) is not found — the page does not reset to the initial upload form state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>Test Execution Data</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>Execution Status</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>Tested By</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>Remarks</t>
-        </is>
-      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Upload a text file successfully shows File Uploaded confirmation</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a text file (e.g., 'test-file.txt') using the file input
+3. Click the Upload button</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-001</t>
+          <t>TC-UPLOAD-003</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1208,13 +1223,14 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Verify page load shows empty file input and no upload confirmation</t>
+          <t>Upload a markdown file successfully shows File Uploaded confirmation</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Inspect the page content</t>
+2. Select a markdown file (e.g., 'CLAUDE.md') using the file input
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -1242,7 +1258,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-002</t>
+          <t>TC-UPLOAD-004</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -1252,28 +1268,29 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Verify instructional text and page structural elements</t>
+          <t>Upload a PNG image file successfully</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Inspect the page for instructional content and structural elements</t>
+2. Select a PNG file (e.g., 'test-image.png') using the file input
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Instructional text about choosing a file and uploading is visible on the page.</t>
+          <t>All assertions pass</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>getByText('Choose a file on your computer') times out after 10 seconds — the expected instructional text is not present in the DOM.</t>
+          <t>All assertions passed</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -1281,16 +1298,12 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>Instructional text 'Choose a file on your computer' not found on upload page</t>
-        </is>
-      </c>
+      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-003</t>
+          <t>TC-UPLOAD-005</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -1300,14 +1313,14 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Upload a single .txt file and verify confirmation view</t>
+          <t>Upload a JSON file successfully</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test .txt file using the file input (id="file-upload")
-3. Click the "Upload" button (id="file-submit")</t>
+2. Select a JSON file (e.g., 'package.json') using the file input
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -1335,7 +1348,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-004</t>
+          <t>TC-UPLOAD-006</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -1345,14 +1358,14 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Upload a .png file and verify filename displayed correctly</t>
+          <t>Upload a PDF file successfully</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test .png file using the file input
-3. Click the "Upload" button</t>
+2. Select a PDF file (e.g., 'document.pdf') using the file input
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -1380,7 +1393,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-005</t>
+          <t>TC-UPLOAD-007</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -1390,14 +1403,14 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Upload a .json file and verify filename displayed correctly</t>
+          <t>Upload file with spaces in name preserves exact filename</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test .json file using the file input
-3. Click the "Upload" button</t>
+2. Select a file named 'my file.txt' (contains spaces)
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -1425,7 +1438,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-006</t>
+          <t>TC-UPLOAD-008</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1435,14 +1448,14 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Upload a .pdf file and verify filename displayed correctly</t>
+          <t>Upload file with parentheses in name preserves exact filename</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test .pdf file using the file input
-3. Click the "Upload" button</t>
+2. Select a file named 'file (1).txt' (contains parentheses)
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -1470,7 +1483,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-007</t>
+          <t>TC-UPLOAD-009</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1480,14 +1493,14 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Upload file with spaces in name and verify exact filename displayed</t>
+          <t>Upload file with spaces and parentheses preserves exact filename</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file with spaces in its name (e.g., "my test file.txt")
-3. Click the "Upload" button</t>
+2. Select a file named 'my file (1).txt' (contains both spaces and parentheses)
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -1515,7 +1528,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-008</t>
+          <t>TC-UPLOAD-010</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -1525,14 +1538,14 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Upload file with spaces and parentheses and verify exact filename displayed</t>
+          <t>Upload file with hyphens and underscores in name</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file with spaces and parentheses in its name (e.g., "my file (1).txt")
-3. Click the "Upload" button</t>
+2. Select a file named 'test_file-name.txt' (contains underscore and hyphen)
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -1560,7 +1573,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-009</t>
+          <t>TC-UPLOAD-011</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -1570,14 +1583,13 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Upload file with hyphens and underscores in name</t>
+          <t>Clicking Upload without selecting a file shows Internal Server Error</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file with hyphens and underscores (e.g., "test-file_01.txt")
-3. Click the "Upload" button</t>
+2. Click the Upload button without selecting any file</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -1605,7 +1617,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-010</t>
+          <t>TC-UPLOAD-012</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -1615,14 +1627,14 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Upload file with mixed special characters</t>
+          <t>File input accepts file selection via browser dialog</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file with multiple special characters (e.g., "test file (v2.1) [final].txt")
-3. Click the "Upload" button</t>
+2. Select a file using the file input via Playwright's setInputFiles API
+3. Verify the file input reflects the selection before submission</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -1650,7 +1662,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-011</t>
+          <t>TC-UPLOAD-013</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -1660,13 +1672,15 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Click Upload with no file selected and verify behavior</t>
+          <t>Selecting then clearing a file leaves input empty and submit fails</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Click the "Upload" button without selecting a file</t>
+2. Select a file (e.g., 'test.txt')
+3. Clear the file selection (setInputFiles with empty array)
+4. Click the Upload button</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -1694,7 +1708,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-012</t>
+          <t>TC-UPLOAD-014</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1704,15 +1718,14 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Select file, clear selection, then click Upload</t>
+          <t>After successful upload, navigating back to /upload resets to initial state</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file using the file input
-3. Clear the file selection by setting the input to empty
-4. Click the "Upload" button</t>
+2. Select a file (e.g., 'reset-test.txt') and click Upload
+3. Navigate back to https://the-internet.herokuapp.com/upload (fresh page load)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -1740,7 +1753,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-013</t>
+          <t>TC-UPLOAD-015</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1750,14 +1763,15 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Upload file with very long filename</t>
+          <t>Multiple uploads in sequence each show correct filename</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
           <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a test file with a very long filename (200+ characters)
-3. Click the "Upload" button</t>
+2. Upload 'first-file.txt'
+3. Navigate back to https://the-internet.herokuapp.com/upload
+4. Upload 'second-file.json'</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -1785,7 +1799,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-014</t>
+          <t>TC-UPLOAD-016</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -1795,15 +1809,13 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Upload same file twice in succession</t>
+          <t>Refreshing the page after upload resets state</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select and upload a test file (e.g., "test-file.txt")
-3. Navigate back to https://the-internet.herokuapp.com/upload
-4. Select and upload the same file again</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload and upload 'refresh-test.txt'
+2. Refresh the page (page.reload())</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -1827,100 +1839,6 @@
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-015</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Navigate back to upload page after successful upload resets state</t>
-        </is>
-      </c>
-      <c r="D85" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select and upload a test file
-3. Navigate to https://the-internet.herokuapp.com/upload (fresh page load)</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-016</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Reload confirmation page returns to initial upload state</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select and upload a test file
-3. Reload/refresh the current page</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Page returns to the initial upload state with 'File Uploader' heading visible and empty file input.</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>After page reload, getByRole('heading', { name: 'File Uploader' }) is not found — the page does not reset to the initial upload form state.</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>Reloading confirmation page does not return to initial upload state</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
chore(pipeline): mark single-file-upload-flow complete --   16 passed (11.6s)
</commit_message>
<xml_diff>
--- a/reports/single-file-upload-flow-test-execution-report.xlsx
+++ b/reports/single-file-upload-flow-test-execution-report.xlsx
@@ -719,7 +719,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Internet - File Upload Test Execution Report</t>
+          <t>The Internet - File Uploader Test Execution Report</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The Internet - File Upload</t>
+          <t>The Internet - File Uploader</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Validate the end-to-end classic HTML file-input upload flow on the-internet.herokuapp.com/upload, covering successful uploads across multiple file types, filename preservation with special characters, negative cases (submitting without a file), and correct page state reset between uploads.</t>
+          <t>Validate the classic file-input upload flow on the File Uploader page end-to-end, covering initial page state, successful uploads across multiple file types, special-character filename preservation, negative cases (no file selected), and state reset after upload, to catch regressions without manual re-testing.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>All 16 test cases passed across 6 use-case groups (Initial Page State, Happy Path Upload, Multiple File Types, Special Characters in Filename, Negative and Edge Cases, State Reset After Upload) with a 100% success rate in 0.4 minutes. No defects were recorded. The suite confirmed that PNG, JSON, PDF, text, and markdown files all upload successfully, filenames with spaces, parentheses, hyphens, and underscores are preserved exactly, and the page correctly resets state after navigation or refresh.</t>
+          <t>All 16 test cases passed across 6 use-case groups (Initial Page State, Successful Upload, File Type Variants, Special Characters in Filenames, Negative/Edge Cases, and State Reset) with a 100% success rate in 0.2 minutes on Chromium. No defects were recorded. The application correctly preserves filenames with spaces, parentheses, brackets, hyphens, and underscores, and properly returns an Internal Server Error when no file is selected.</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>No corrective action is needed — the suite is fully green with zero defects. Consider expanding coverage in future iterations to include drag-and-drop upload (currently out of scope), large file behavior, and additional browsers beyond Chromium if cross-browser confidence is desired.</t>
+          <t>No corrective action is needed as all tests passed and no defects were found. Consider expanding coverage in future iterations to include drag-and-drop upload behavior, large file uploads, and cross-browser validation if those scenarios become acceptance criteria.</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>The single-file-upload-flow suite is fully passing and the File Upload feature behaves correctly across all tested scenarios, confirming regression-safe status for this feature area.</t>
+          <t>The single-file-upload-flow suite is fully green with 16/16 tests passing and zero defects, confirming the File Uploader feature meets all specified acceptance criteria.</t>
         </is>
       </c>
     </row>
@@ -1129,18 +1129,18 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Verify initial page load state shows file input and no confirmation</t>
+          <t>Verify initial page load state shows File Uploader heading, empty file input, and no confirmation</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Verify the initial page content</t>
+          <t>1. Navigate to the File Uploader page (https://the-internet.herokuapp.com/upload)
+2. Inspect the page content</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -1173,19 +1173,19 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Upload a text file successfully shows File Uploaded confirmation</t>
+          <t>Upload a simple text file and verify confirmation with exact filename</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a text file (e.g., 'test-file.txt') using the file input
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a simple text file (e.g., "test.txt") in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -1218,19 +1218,19 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Upload a markdown file successfully shows File Uploaded confirmation</t>
+          <t>Upload a PNG image file and verify confirmation with exact filename</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a markdown file (e.g., 'CLAUDE.md') using the file input
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a PNG image file (e.g., "image.png") in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -1263,19 +1263,19 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Upload a PNG image file successfully</t>
+          <t>Upload a JSON file and verify confirmation with exact filename</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a PNG file (e.g., 'test-image.png') using the file input
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a JSON file (e.g., "data.json") in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -1308,19 +1308,19 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Upload a JSON file successfully</t>
+          <t>Upload a PDF file and verify confirmation with exact filename</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a JSON file (e.g., 'package.json') using the file input
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a PDF file (e.g., "document.pdf") in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -1353,19 +1353,19 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Upload a PDF file successfully</t>
+          <t>Upload file with spaces in filename and verify exact filename preservation</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a PDF file (e.g., 'document.pdf') using the file input
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file with spaces in the name (e.g., "my test file.txt") in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -1398,19 +1398,19 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Upload file with spaces in name preserves exact filename</t>
+          <t>Upload file with parentheses in filename and verify exact filename preservation</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file named 'my file.txt' (contains spaces)
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file with parentheses in the name (e.g., "file(1).txt") in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -1443,19 +1443,19 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Upload file with parentheses in name preserves exact filename</t>
+          <t>Upload file with multiple special characters in filename and verify exact filename preservation</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file named 'file (1).txt' (contains parentheses)
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file with multiple special characters in the name (e.g., "my_file (copy) [2].txt") in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -1488,19 +1488,19 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Upload file with spaces and parentheses preserves exact filename</t>
+          <t>Clicking Upload with no file selected results in Internal Server Error</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file named 'my file (1).txt' (contains both spaces and parentheses)
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Do NOT select any file in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -1533,19 +1533,19 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Upload file with hyphens and underscores in name</t>
+          <t>Verify upload with no file selected does not show confirmation elements</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file named 'test_file-name.txt' (contains underscore and hyphen)
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Do NOT select any file in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -1578,18 +1578,20 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Clicking Upload without selecting a file shows Internal Server Error</t>
+          <t>After successful upload, navigating back to upload page resets to initial empty state</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Click the Upload button without selecting any file</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file (e.g., "test.txt") in the file input
+3. Click the "Upload" submit button
+4. Navigate back to the File Uploader page (https://the-internet.herokuapp.com/upload)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -1622,19 +1624,18 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>File input accepts file selection via browser dialog</t>
+          <t>Verify confirmation view URL remains the same after successful upload</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file using the file input via Playwright's setInputFiles API
-3. Verify the file input reflects the selection before submission</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file (e.g., "test.txt") and click Upload</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -1667,20 +1668,19 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Selecting then clearing a file leaves input empty and submit fails</t>
+          <t>Upload file with hyphen and underscore in filename</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file (e.g., 'test.txt')
-3. Clear the file selection (setInputFiles with empty array)
-4. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file with hyphens and underscores (e.g., "test-file_01.txt") in the file input
+3. Click the "Upload" submit button</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -1713,19 +1713,19 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>After successful upload, navigating back to /upload resets to initial state</t>
+          <t>Verify file input accepts any file type (no extension restriction)</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file (e.g., 'reset-test.txt') and click Upload
-3. Navigate back to https://the-internet.herokuapp.com/upload (fresh page load)</t>
+          <t>1. Navigate to the File Uploader page
+2. Inspect the file input element
+3. Select a file with an uncommon extension (e.g., "data.csv") and click Upload</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -1758,20 +1758,18 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Multiple uploads in sequence each show correct filename</t>
+          <t>Verify file input is not marked as required</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Upload 'first-file.txt'
-3. Navigate back to https://the-internet.herokuapp.com/upload
-4. Upload 'second-file.json'</t>
+          <t>1. Navigate to the File Uploader page
+2. Inspect the file input element's attributes</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -1804,18 +1802,19 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Refreshing the page after upload resets state</t>
+          <t>Sequential uploads — upload one file, reset, upload a different file</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload and upload 'refresh-test.txt'
-2. Refresh the page (page.reload())</t>
+          <t>1. Navigate to the File Uploader page and upload "first.txt"
+2. Navigate back to the upload page
+3. Select a different file (e.g., "second.txt") and click Upload</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">

</xml_diff>

<commit_message>
chore(pipeline): mark single-file-upload-flow complete --   18 passed (14.1s)
</commit_message>
<xml_diff>
--- a/reports/single-file-upload-flow-test-execution-report.xlsx
+++ b/reports/single-file-upload-flow-test-execution-report.xlsx
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -775,7 +775,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Validate the classic file-input upload flow on the File Uploader page end-to-end, covering initial page state, successful uploads across multiple file types, special-character filename preservation, negative cases (no file selected), and state reset after upload, to catch regressions without manual re-testing.</t>
+          <t>Validate the classic HTML file-input upload flow on the File Uploader page end-to-end, ensuring filename preservation across file types and special characters, correct error behavior when no file is selected, and proper state reset between uploads.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>All 16 test cases passed across 6 use-case groups (Initial Page State, Successful Upload, File Type Variants, Special Characters in Filenames, Negative/Edge Cases, and State Reset) with a 100% success rate in 0.2 minutes on Chromium. No defects were recorded. The application correctly preserves filenames with spaces, parentheses, brackets, hyphens, and underscores, and properly returns an Internal Server Error when no file is selected.</t>
+          <t>All 18 test cases passed with a 100% success rate across 9 use-case groups (Initial Page State, Basic Upload Happy Path, Multiple File Types, Special Character Filenames, No File Selected, Sequential Uploads, State Reset, File Input Behavior, and Boundary Cases) in 0.24 minutes on Chromium. No defects were recorded. The application correctly handles .txt, .png, .json, and .pdf uploads, preserves filenames with spaces, parentheses, dashes, underscores, and multiple dots, displays very long and extensionless filenames correctly, and returns an Internal Server Error when no file is selected.</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>No corrective action is needed as all tests passed and no defects were found. Consider expanding coverage in future iterations to include drag-and-drop upload behavior, large file uploads, and cross-browser validation if those scenarios become acceptance criteria.</t>
+          <t>No corrective action is needed as all tests passed and no defects were found. Consider expanding coverage in future iterations to include the drag-and-drop upload widget (currently out of scope) and cross-browser validation beyond Chromium if those scenarios become acceptance criteria.</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>The single-file-upload-flow suite is fully green with 16/16 tests passing and zero defects, confirming the File Uploader feature meets all specified acceptance criteria.</t>
+          <t>The single-file-upload-flow suite is fully green with 18/18 tests passing and zero defects, confirming the File Uploader feature meets all specified acceptance criteria across all tested scenarios.</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39">
@@ -1129,17 +1129,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Verify initial page load state shows File Uploader heading, empty file input, and no confirmation</t>
+          <t>Verify initial page state shows empty file input and no confirmation</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page (https://the-internet.herokuapp.com/upload)
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
 2. Inspect the page content</t>
         </is>
       </c>
@@ -1173,19 +1173,19 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Upload a simple text file and verify confirmation with exact filename</t>
+          <t>Basic upload with .txt file succeeds and shows confirmation</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a simple text file (e.g., "test.txt") in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a .txt file in the file input (e.g., 'test.txt')
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -1218,19 +1218,20 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Upload a PNG image file and verify confirmation with exact filename</t>
+          <t>Upload confirmation displays exact uploaded filename</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a PNG image file (e.g., "image.png") in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a .txt file with a unique name (e.g., 'my-test-file.txt')
+3. Click the Upload button
+4. Verify the displayed filename</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -1263,19 +1264,19 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Upload a JSON file and verify confirmation with exact filename</t>
+          <t>Upload .png image file succeeds and shows correct filename</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a JSON file (e.g., "data.json") in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a .png file in the file input (e.g., 'image.png')
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -1308,19 +1309,19 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Upload a PDF file and verify confirmation with exact filename</t>
+          <t>Upload .json file succeeds and shows correct filename</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a PDF file (e.g., "document.pdf") in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a .json file in the file input (e.g., 'data.json')
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -1353,19 +1354,19 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Upload file with spaces in filename and verify exact filename preservation</t>
+          <t>Upload .pdf file succeeds and shows correct filename</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a file with spaces in the name (e.g., "my test file.txt") in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a .pdf file in the file input (e.g., 'document.pdf')
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -1398,19 +1399,19 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Upload file with parentheses in filename and verify exact filename preservation</t>
+          <t>Filename with spaces preserved exactly on confirmation</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a file with parentheses in the name (e.g., "file(1).txt") in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file whose name contains spaces (e.g., 'my test file.txt')
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -1443,19 +1444,19 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Upload file with multiple special characters in filename and verify exact filename preservation</t>
+          <t>Filename with parentheses and spaces preserved exactly</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a file with multiple special characters in the name (e.g., "my_file (copy) [2].txt") in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file with parentheses in the name (e.g., 'my file (1).txt')
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -1488,19 +1489,19 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Clicking Upload with no file selected results in Internal Server Error</t>
+          <t>Filename with dashes and underscores preserved exactly</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Do NOT select any file in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file with dashes and underscores (e.g., 'test_file-v2.txt')
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -1533,19 +1534,19 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Verify upload with no file selected does not show confirmation elements</t>
+          <t>Filename with dots (multiple extensions pattern) preserved exactly</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Do NOT select any file in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file with multiple dots in the name (e.g., 'backup.2024.01.15.tar.gz')
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -1578,20 +1579,18 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>After successful upload, navigating back to upload page resets to initial empty state</t>
+          <t>Clicking Upload with no file selected results in server error</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a file (e.g., "test.txt") in the file input
-3. Click the "Upload" submit button
-4. Navigate back to the File Uploader page (https://the-internet.herokuapp.com/upload)</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Click the Upload button without selecting any file</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -1624,18 +1623,20 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Verify confirmation view URL remains the same after successful upload</t>
+          <t>Multiple sequential uploads each show their own correct filename</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a file (e.g., "test.txt") and click Upload</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a .txt file (e.g., 'first.txt') and click Upload
+3. Navigate back to https://the-internet.herokuapp.com/upload
+4. Select a different file (e.g., 'second.png') and click Upload</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -1668,19 +1669,19 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Upload file with hyphen and underscore in filename</t>
+          <t>After successful upload, navigating back resets page to initial state</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Select a file with hyphens and underscores (e.g., "test-file_01.txt") in the file input
-3. Click the "Upload" submit button</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file (e.g., 'test.txt') and click Upload
+3. Navigate back to https://the-internet.herokuapp.com/upload</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -1713,19 +1714,20 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Verify file input accepts any file type (no extension restriction)</t>
+          <t>File input accepts selection change before upload</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Inspect the file input element
-3. Select a file with an uncommon extension (e.g., "data.csv") and click Upload</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a .txt file (e.g., 'original.txt')
+3. Before clicking Upload, select a different file (e.g., 'replacement.json')
+4. Click the Upload button</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -1758,18 +1760,19 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Verify file input is not marked as required</t>
+          <t>Upload button remains enabled throughout interaction</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page
-2. Inspect the file input element's attributes</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file in the file input
+3. Clear the file selection (select then cancel file dialog)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -1802,19 +1805,19 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Sequential uploads — upload one file, reset, upload a different file</t>
+          <t>Page URL remains /upload throughout the upload flow</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to the File Uploader page and upload "first.txt"
-2. Navigate back to the upload page
-3. Select a different file (e.g., "second.txt") and click Upload</t>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file and click Upload
+3. Navigate back to /upload</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -1838,6 +1841,96 @@
         </is>
       </c>
       <c r="I84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-017</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Large filename (long string) is displayed completely</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file with a very long filename (e.g., 'this_is_a_very_long_filename_that_contains_many_characters_and_should_still_be_displayed_correctly.txt' - 100+ chars)
+3. Click the Upload button</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-018</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>File with no extension (extensionless filename) uploads successfully</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to https://the-internet.herokuapp.com/upload
+2. Select a file with no extension (e.g., filename 'README' or 'Makefile')
+3. Click the Upload button</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
chore(pipeline): mark single-file-upload-flow complete --   7 failed   13 passed (2.8m)
</commit_message>
<xml_diff>
--- a/reports/single-file-upload-flow-test-execution-report.xlsx
+++ b/reports/single-file-upload-flow-test-execution-report.xlsx
@@ -702,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -775,7 +775,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Validate the classic HTML file-input upload flow on the File Uploader page end-to-end, ensuring filename preservation across file types and special characters, correct error behavior when no file is selected, and proper state reset between uploads.</t>
+          <t>Verify the end-to-end single-file upload workflow — file selection, form submission, success-page confirmation with correct filename, navigation state reset, and empty-submission handling — on the-internet.herokuapp.com/upload, providing automated regression coverage that catches regressions without manual re-testing.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>All 18 test cases passed with a 100% success rate across 9 use-case groups (Initial Page State, Basic Upload Happy Path, Multiple File Types, Special Character Filenames, No File Selected, Sequential Uploads, State Reset, File Input Behavior, and Boundary Cases) in 0.24 minutes on Chromium. No defects were recorded. The application correctly handles .txt, .png, .json, and .pdf uploads, preserves filenames with spaces, parentheses, dashes, underscores, and multiple dots, displays very long and extensionless filenames correctly, and returns an Internal Server Error when no file is selected.</t>
+          <t>Of 20 test cases executed, 13 passed (65%) and 7 failed across 5 distinct defects. The highest-severity issue (BUG-003, High) is that submitting the upload form with no file selected returns an HTTP 500 Internal Server Error instead of a user-friendly validation message, affecting TC-UPLOAD-009 and TC-UPLOAD-010. Two medium-severity defects were found: BUG-002 shows that back-navigation from the success page does not clear the file input state (TC-UPLOAD-007, TC-UPLOAD-008), and BUG-005 reveals the form element lacks the expected id attribute 'file-upload-form' causing TC-UPLOAD-017 to fail on locator timeout. Two low-severity issues (BUG-001, BUG-004) are test-implementation mismatches rather than application bugs — the instructional text wording differs from what the test asserts, and the multi-file enforcement test triggers a Playwright error instead of asserting the 'multiple' attribute absence.</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>No corrective action is needed as all tests passed and no defects were found. Consider expanding coverage in future iterations to include the drag-and-drop upload widget (currently out of scope) and cross-browser validation beyond Chromium if those scenarios become acceptance criteria.</t>
+          <t>Fix the application's empty-submission handling (BUG-003) as a priority — an HTTP 500 on a foreseeable user action is a genuine server-side defect. For BUG-002, investigate whether the back-navigation state retention is intended browser caching behavior or an application bug, and adjust the test expectation or file a fix accordingly. For the two low-severity test-implementation issues (BUG-001 and BUG-004), update the test locators and assertion approach to match the actual page content: use the real instructional text wording and assert the absence of the 'multiple' attribute rather than calling setInputFiles with two files. For BUG-005, inspect the actual form element's id and update the locator in the page object.</t>
         </is>
       </c>
     </row>
@@ -855,7 +855,7 @@
     <row r="21" ht="45" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>The single-file-upload-flow suite is fully green with 18/18 tests passing and zero defects, confirming the File Uploader feature meets all specified acceptance criteria across all tested scenarios.</t>
+          <t>The suite's core happy-path upload flows (text, image, special-character and long filenames, edge-case filenames) all pass reliably, confirming the primary upload functionality is solid. The 65% pass rate is driven by a mix of one genuine application defect (empty-submission 500 error) and test-implementation gaps (incorrect locators and assertion strategies) that should be straightforward to resolve.</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39">
@@ -1000,7 +1000,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40">
@@ -1067,321 +1067,279 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>BUG-001</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Instructional text locator mismatch — 'Choose a file on your computer' not found on page</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>QA Automation</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>getByText('Choose a file on your computer') finds no matching element; the page uses different instructional wording than the test expects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>BUG-002</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Back-navigation from success page does not clear file input state</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>QA Automation</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>File input retains the previously selected file path (e.g. 'C:\fakepath\first-file.txt') after back-navigation; toHaveValue('') times out.</t>
+        </is>
+      </c>
+    </row>
     <row r="67">
-      <c r="A67" s="5" t="inlineStr">
-        <is>
-          <t>Test Execution Data</t>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BUG-003</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Submitting upload form with no file selected returns HTTP 500 Internal Server Error</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>QA Automation</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Page navigates to an 'Internal Server Error' (HTTP 500) page instead of showing a validation message.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>Test Steps</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>Execution Status</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>Tested By</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>Remarks</t>
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>BUG-004</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Test attempts setInputFiles with multiple files on non-multiple file input — Playwright rejects</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>QA Automation</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Playwright throws 'Non-multiple file input can only accept single file' because setInputFiles([file1, file2]) is called on an input without the 'multiple' attribute — the enforcement works but the test approach triggers an error instead of asserting the attribute.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-001</t>
+          <t>BUG-005</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Verify initial page state shows empty file input and no confirmation</t>
-        </is>
-      </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Inspect the page content</t>
+          <t>Form element locator '#file-upload-form' not found — ID does not exist on the form</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>QA Automation</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-002</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Basic upload with .txt file succeeds and shows confirmation</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a .txt file in the file input (e.g., 'test.txt')
-3. Click the Upload button</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-003</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Upload confirmation displays exact uploaded filename</t>
-        </is>
-      </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a .txt file with a unique name (e.g., 'my-test-file.txt')
-3. Click the Upload button
-4. Verify the displayed filename</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr"/>
+          <t>locator('#file-upload-form') times out after 10 seconds — the form element on the page does not have id='file-upload-form'.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-004</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Upload .png image file succeeds and shows correct filename</t>
-        </is>
-      </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a .png file in the file input (e.g., 'image.png')
-3. Click the Upload button</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr"/>
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Test Execution Data</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>TC-UPLOAD-005</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Upload .json file succeeds and shows correct filename</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a .json file in the file input (e.g., 'data.json')
-3. Click the Upload button</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>All assertions pass</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>All assertions passed</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>PASSED</t>
-        </is>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>Playwright Automation</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Execution Status</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Tested By</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-006</t>
+          <t>TC-UPLOAD-001</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Upload .pdf file succeeds and shows correct filename</t>
+          <t>Verify page loads with upload form elements present</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a .pdf file in the file input (e.g., 'document.pdf')
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>Instructional text about choosing/dragging a file is visible on the page.</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>getByText('Choose a file on your computer') finds no matching element; the page uses different instructional wording than the test expects.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -1389,29 +1347,32 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Instructional text locator mismatch — 'Choose a file on your computer' not found on page</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-007</t>
+          <t>TC-UPLOAD-002</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Filename with spaces preserved exactly on confirmation</t>
+          <t>Verify file input control displays no file selected initially</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file whose name contains spaces (e.g., 'my test file.txt')
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Inspect the file input control</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -1439,23 +1400,23 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-008</t>
+          <t>TC-UPLOAD-003</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Filename with parentheses and spaces preserved exactly</t>
+          <t>Upload a valid text file and verify success page</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file with parentheses in the name (e.g., 'my file (1).txt')
+          <t>1. Navigate to the File Uploader page
+2. Select a valid text file via the file input control (e.g., 'test-upload.txt')
 3. Click the Upload button</t>
         </is>
       </c>
@@ -1484,23 +1445,23 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-009</t>
+          <t>TC-UPLOAD-004</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Filename with dashes and underscores preserved exactly</t>
+          <t>Upload a valid image file (PNG) and verify success page</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file with dashes and underscores (e.g., 'test_file-v2.txt')
+          <t>1. Navigate to the File Uploader page
+2. Select a valid PNG image file via the file input control (e.g., 'test-image.png')
 3. Click the Upload button</t>
         </is>
       </c>
@@ -1529,23 +1490,23 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-010</t>
+          <t>TC-UPLOAD-005</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Filename with dots (multiple extensions pattern) preserved exactly</t>
+          <t>Upload a file with spaces and special characters in filename</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file with multiple dots in the name (e.g., 'backup.2024.01.15.tar.gz')
+          <t>1. Navigate to the File Uploader page
+2. Select a file with spaces/special characters in name (e.g., 'My Test File (1).txt')
 3. Click the Upload button</t>
         </is>
       </c>
@@ -1574,23 +1535,24 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-011</t>
+          <t>TC-UPLOAD-006</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Clicking Upload with no file selected results in server error</t>
+          <t>Upload a file with a long filename</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Click the Upload button without selecting any file</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file with a long filename (e.g., 'this-is-a-very-long-filename-that-exceeds-typical-length-expectations-for-testing-purposes.txt', 100+ characters)
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -1618,40 +1580,42 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-012</t>
+          <t>TC-UPLOAD-007</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Multiple sequential uploads each show their own correct filename</t>
+          <t>Upload a second file after a previous successful upload replaces the displayed filename</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a .txt file (e.g., 'first.txt') and click Upload
-3. Navigate back to https://the-internet.herokuapp.com/upload
-4. Select a different file (e.g., 'second.png') and click Upload</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a first file (e.g., 'first-file.txt')
+3. Click the Upload button
+4. Navigate back to the upload form using the browser's back button
+5. Select a second, different file (e.g., 'second-file.txt')
+6. Click the Upload button</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>File input control is in a clean state (empty value) after navigating back from the success page.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>File input retains the previously selected file path (e.g. 'C:\fakepath\first-file.txt') after back-navigation; toHaveValue('') times out.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -1659,44 +1623,48 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Back-navigation from success page does not clear file input state</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-013</t>
+          <t>TC-UPLOAD-008</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>After successful upload, navigating back resets page to initial state</t>
+          <t>Navigating back from success page returns to a clean upload form</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file (e.g., 'test.txt') and click Upload
-3. Navigate back to https://the-internet.herokuapp.com/upload</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file (e.g., 'test-file.txt') and upload it
+3. Click the browser's back button</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>File input control is in a clean state (empty value) after navigating back from the success page.</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>File input retains the previously selected file path (e.g. 'C:\fakepath\first-file.txt') after back-navigation; toHaveValue('') times out.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -1704,45 +1672,47 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Back-navigation from success page does not clear file input state</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-014</t>
+          <t>TC-UPLOAD-009</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>File input accepts selection change before upload</t>
+          <t>Clicking Upload with no file selected displays a validation message (not server error)</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a .txt file (e.g., 'original.txt')
-3. Before clicking Upload, select a different file (e.g., 'replacement.json')
-4. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Click the Upload button without selecting a file</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>A user-friendly validation message is displayed and the user remains on the upload form.</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>Page navigates to an 'Internal Server Error' (HTTP 500) page instead of showing a validation message.</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -1750,44 +1720,49 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Submitting upload form with no file selected returns HTTP 500 Internal Server Error</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-015</t>
+          <t>TC-UPLOAD-010</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Upload button remains enabled throughout interaction</t>
+          <t>Selecting a file then clearing selection before upload</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file in the file input
-3. Clear the file selection (select then cancel file dialog)</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a file via the file input control (e.g., 'test.txt')
+3. Clear the file selection (click 'Choose File' again and cancel without selecting, or programmatically clear if the UI allows)
+4. Click the Upload button</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>All assertions pass</t>
+          <t>A user-friendly validation message is displayed and the user remains on the upload form.</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>All assertions passed</t>
+          <t>Page navigates to an 'Internal Server Error' (HTTP 500) page instead of showing a validation message.</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>FAILED</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -1795,29 +1770,33 @@
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Submitting upload form with no file selected returns HTTP 500 Internal Server Error</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-016</t>
+          <t>TC-UPLOAD-011</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Page URL remains /upload throughout the upload flow</t>
+          <t>File input control accepts and uploads a zero-byte (empty) file</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file and click Upload
-3. Navigate back to /upload</t>
+          <t>1. Navigate to the File Uploader page
+2. Select a zero-byte file (e.g., 'empty.txt' with 0 bytes)
+3. Click the Upload button</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -1845,24 +1824,23 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TC-UPLOAD-017</t>
+          <t>TC-UPLOAD-012</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Large filename (long string) is displayed completely</t>
+          <t>Selecting a file via file input populates the control with the filename before submission</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file with a very long filename (e.g., 'this_is_a_very_long_filename_that_contains_many_characters_and_should_still_be_displayed_correctly.txt' - 100+ chars)
-3. Click the Upload button</t>
+          <t>1. Navigate to the File Uploader page
+2. Click the 'Choose File' button and select a file (e.g., 'sample.txt') from the file picker dialog</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -1890,47 +1868,368 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>TC-UPLOAD-013</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Replacing a selected file with a different file updates the file input display</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to the File Uploader page
+2. Select a first file (e.g., 'file-one.txt')
+3. Click 'Choose File' again and select a different file (e.g., 'file-two.txt'), replacing the first selection
+4. Click the Upload button</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-014</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>File input control does not accept multiple files simultaneously (single file upload)</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to the File Uploader page
+2. Inspect the file input control's HTML attributes
+3. Attempt to select multiple files via the file picker (Shift+click or Ctrl+click multiple files in the dialog, if the control allows it)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>The file input accepts only a single file (test verifies single-file enforcement).</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Playwright throws 'Non-multiple file input can only accept single file' because setInputFiles([file1, file2]) is called on an input without the 'multiple' attribute — the enforcement works but the test approach triggers an error instead of asserting the attribute.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Test attempts setInputFiles with multiple files on non-multiple file input — Playwright rejects</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-015</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>File input control has correct HTML attributes (id, name, type)</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to the File Uploader page
+2. Inspect the file input control's HTML attributes</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-016</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Upload button has correct attributes and is clickable before file selection</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to the File Uploader page
+2. Inspect the Upload button's attributes</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-017</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Form element has correct action and method attributes</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to the File Uploader page
+2. Inspect the form element's attributes</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Form element is found and its action/method/enctype attributes are verified.</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>locator('#file-upload-form') times out after 10 seconds — the form element on the page does not have id='file-upload-form'.</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Form element locator '#file-upload-form' not found — ID does not exist on the form</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
           <t>TC-UPLOAD-018</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>File with no extension (extensionless filename) uploads successfully</t>
-        </is>
-      </c>
-      <c r="D86" s="4" t="inlineStr">
-        <is>
-          <t>1. Navigate to https://the-internet.herokuapp.com/upload
-2. Select a file with no extension (e.g., filename 'README' or 'Makefile')
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Upload a file with no extension</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to the File Uploader page
+2. Select a file with no file extension (e.g., filename is just 'testfile' with no dot or extension)
 3. Click the Upload button</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>All assertions pass</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>All assertions passed</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
+      <c r="G91" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="H91" t="inlineStr">
         <is>
           <t>Playwright Automation</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-019</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Upload a file with multiple dots in the filename</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to the File Uploader page
+2. Select a file with multiple dots (e.g., 'my.test.file.backup.txt')
+3. Click the Upload button</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>TC-UPLOAD-020</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Upload a file with unicode characters in the filename</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>1. Navigate to the File Uploader page
+2. Select a file with unicode/non-ASCII characters (e.g., 'tëst-fîlé.txt')
+3. Click the Upload button</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>All assertions pass</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>All assertions passed</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Playwright Automation</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>